<commit_message>
yang sebelumnya error, ini dah bener
</commit_message>
<xml_diff>
--- a/monitoring_weighted_similarity.xlsx
+++ b/monitoring_weighted_similarity.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M121"/>
+  <dimension ref="A1:M122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3298,47 +3298,45 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>GAMMA RAYA, CV</t>
+          <t>SEXY ROAD INDO, CV</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>7571</t>
+          <t>7501</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Jalan Rusli Datau 1 Perumahan Alya III Blok B Nomor 2</t>
+          <t>Perum Asabri Blok E/03</t>
         </is>
       </c>
       <c r="F54" t="n">
-        <v>153</v>
+        <v>0</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>GAMMA RAYA, CV</t>
+          <t>MARKA INDAH, CV</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>7571</t>
+          <t>7501</t>
         </is>
       </c>
       <c r="I54" t="n">
-        <v>100</v>
+        <v>60.60606060606061</v>
       </c>
       <c r="J54" t="n">
         <v>100</v>
       </c>
-      <c r="K54" t="n">
-        <v>92.92929292929293</v>
-      </c>
+      <c r="K54" t="inlineStr"/>
       <c r="L54" t="n">
-        <v>94.72186655285246</v>
+        <v>67.76859504132231</v>
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>DROP</t>
+          <t>INSERT</t>
         </is>
       </c>
     </row>
@@ -3353,45 +3351,47 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>TRI BAROKAH PERKASA, PT</t>
+          <t>GAMMA RAYA, CV</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>7503</t>
+          <t>7571</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Jl. Kasmat Lahay</t>
+          <t>Jalan Rusli Datau 1 Perumahan Alya III Blok B Nomor 2</t>
         </is>
       </c>
       <c r="F55" t="n">
-        <v>1191</v>
+        <v>153</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>PUTRA MITRA PERKASA, CV</t>
+          <t>GAMMA RAYA, CV</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>7503</t>
+          <t>7571</t>
         </is>
       </c>
       <c r="I55" t="n">
-        <v>65.21739130434783</v>
+        <v>100</v>
       </c>
       <c r="J55" t="n">
         <v>100</v>
       </c>
-      <c r="K55" t="inlineStr"/>
+      <c r="K55" t="n">
+        <v>92.92929292929293</v>
+      </c>
       <c r="L55" t="n">
-        <v>70.37037037037037</v>
+        <v>94.72186655285246</v>
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>INSERT</t>
+          <t>DROP</t>
         </is>
       </c>
     </row>
@@ -3406,41 +3406,41 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>INDO KONSTRUKSI PERSADA, PT</t>
+          <t>TRI BAROKAH PERKASA, PT</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>7501</t>
+          <t>7503</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Jalan Sun Ismail Perum Latoro</t>
+          <t>Jl. Kasmat Lahay</t>
         </is>
       </c>
       <c r="F56" t="n">
-        <v>207</v>
+        <v>1191</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>LUTSIR PERSADA JAYA, PT</t>
+          <t>PUTRA MITRA PERKASA, CV</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>7501</t>
+          <t>7503</t>
         </is>
       </c>
       <c r="I56" t="n">
-        <v>60</v>
+        <v>65.21739130434783</v>
       </c>
       <c r="J56" t="n">
         <v>100</v>
       </c>
       <c r="K56" t="inlineStr"/>
       <c r="L56" t="n">
-        <v>65.16129032258064</v>
+        <v>70.37037037037037</v>
       </c>
       <c r="M56" t="inlineStr">
         <is>
@@ -3459,41 +3459,41 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>HAVANA TUNAS GEMILANG, PT</t>
+          <t>INDO KONSTRUKSI PERSADA, PT</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>7504</t>
+          <t>7501</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>JALAN DIPENOGORO BLOK PLAN PERKANTORAN MARISA</t>
+          <t>Jalan Sun Ismail Perum Latoro</t>
         </is>
       </c>
       <c r="F57" t="n">
-        <v>1481</v>
+        <v>207</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>RISKY MAHARANI ENERGI, PT</t>
+          <t>LUTSIR PERSADA JAYA, PT</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>7504</t>
+          <t>7501</t>
         </is>
       </c>
       <c r="I57" t="n">
-        <v>56.00000000000001</v>
+        <v>60</v>
       </c>
       <c r="J57" t="n">
         <v>100</v>
       </c>
       <c r="K57" t="inlineStr"/>
       <c r="L57" t="n">
-        <v>62.06896551724139</v>
+        <v>65.16129032258064</v>
       </c>
       <c r="M57" t="inlineStr">
         <is>
@@ -3512,7 +3512,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>MEGA UTAMA MARISA, CV</t>
+          <t>HAVANA TUNAS GEMILANG, PT</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -3522,15 +3522,15 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>DUSUN BATU PASANG</t>
+          <t>JALAN DIPENOGORO BLOK PLAN PERKANTORAN MARISA</t>
         </is>
       </c>
       <c r="F58" t="n">
-        <v>1426</v>
+        <v>1481</v>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>MULIA MULTI MANDIRI, CV</t>
+          <t>RISKY MAHARANI ENERGI, PT</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -3539,14 +3539,14 @@
         </is>
       </c>
       <c r="I58" t="n">
-        <v>63.63636363636363</v>
+        <v>56.00000000000001</v>
       </c>
       <c r="J58" t="n">
         <v>100</v>
       </c>
       <c r="K58" t="inlineStr"/>
       <c r="L58" t="n">
-        <v>69.45454545454545</v>
+        <v>62.06896551724139</v>
       </c>
       <c r="M58" t="inlineStr">
         <is>
@@ -3565,43 +3565,41 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>ANNISA RAMADHANI PROPERTINDO, PT</t>
+          <t>MEGA UTAMA MARISA, CV</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>7571</t>
+          <t>7504</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Jalan Profesor H.B Jassin Nomor 303</t>
+          <t>DUSUN BATU PASANG</t>
         </is>
       </c>
       <c r="F59" t="n">
-        <v>2035</v>
+        <v>1426</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>POPA EYATO JAYA TAMA, PT</t>
+          <t>MULIA MULTI MANDIRI, CV</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>7571</t>
+          <t>7504</t>
         </is>
       </c>
       <c r="I59" t="n">
-        <v>46.42857142857143</v>
+        <v>63.63636363636363</v>
       </c>
       <c r="J59" t="n">
         <v>100</v>
       </c>
-      <c r="K59" t="n">
-        <v>56.14035087719298</v>
-      </c>
+      <c r="K59" t="inlineStr"/>
       <c r="L59" t="n">
-        <v>54.23417699177521</v>
+        <v>69.45454545454545</v>
       </c>
       <c r="M59" t="inlineStr">
         <is>
@@ -3620,7 +3618,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>NJ GROUP, CV</t>
+          <t>ANNISA RAMADHANI PROPERTINDO, PT</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -3630,15 +3628,15 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Perumahan Awara Karya Blok A.08</t>
+          <t>Jalan Profesor H.B Jassin Nomor 303</t>
         </is>
       </c>
       <c r="F60" t="n">
-        <v>1790</v>
+        <v>2035</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>RIZKIA LESTARI, CV</t>
+          <t>POPA EYATO JAYA TAMA, PT</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -3647,16 +3645,16 @@
         </is>
       </c>
       <c r="I60" t="n">
-        <v>40</v>
+        <v>46.42857142857143</v>
       </c>
       <c r="J60" t="n">
         <v>100</v>
       </c>
       <c r="K60" t="n">
-        <v>75.86206896551724</v>
+        <v>56.14035087719298</v>
       </c>
       <c r="L60" t="n">
-        <v>68.76008804108584</v>
+        <v>54.23417699177521</v>
       </c>
       <c r="M60" t="inlineStr">
         <is>
@@ -3675,41 +3673,43 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>SULTAN JAYA NUSANTARA, CV</t>
+          <t>NJ GROUP, CV</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>7501</t>
+          <t>7571</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Kelurahan Kayumerah</t>
+          <t>Perumahan Awara Karya Blok A.08</t>
         </is>
       </c>
       <c r="F61" t="n">
-        <v>296</v>
+        <v>1790</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>KARYA PATRIOT NUSANTARA, CV</t>
+          <t>RIZKIA LESTARI, CV</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>7501</t>
+          <t>7571</t>
         </is>
       </c>
       <c r="I61" t="n">
-        <v>73.07692307692308</v>
+        <v>40</v>
       </c>
       <c r="J61" t="n">
         <v>100</v>
       </c>
-      <c r="K61" t="inlineStr"/>
+      <c r="K61" t="n">
+        <v>75.86206896551724</v>
+      </c>
       <c r="L61" t="n">
-        <v>76.79045092838197</v>
+        <v>68.76008804108584</v>
       </c>
       <c r="M61" t="inlineStr">
         <is>
@@ -3728,7 +3728,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>INDRA PRAHASTA, CV</t>
+          <t>SULTAN JAYA NUSANTARA, CV</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -3738,15 +3738,15 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Telaga Biru</t>
+          <t>Kelurahan Kayumerah</t>
         </is>
       </c>
       <c r="F62" t="n">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>INKA PRATAMA, CV</t>
+          <t>KARYA PATRIOT NUSANTARA, CV</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -3755,14 +3755,14 @@
         </is>
       </c>
       <c r="I62" t="n">
-        <v>76.47058823529412</v>
+        <v>73.07692307692308</v>
       </c>
       <c r="J62" t="n">
         <v>100</v>
       </c>
       <c r="K62" t="inlineStr"/>
       <c r="L62" t="n">
-        <v>80.74866310160428</v>
+        <v>76.79045092838197</v>
       </c>
       <c r="M62" t="inlineStr">
         <is>
@@ -3781,41 +3781,41 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>MOTIKACI FAMILY GROUP, CV</t>
+          <t>INDRA PRAHASTA, CV</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>7505</t>
+          <t>7501</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Dusun Pasar Lama, Desa Moluo, Kecamatan Kwandang, Kabupaten Gorontalo Utara.</t>
+          <t>Telaga Biru</t>
         </is>
       </c>
       <c r="F63" t="n">
-        <v>1597</v>
+        <v>292</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>TIRTA TARUNA, CV</t>
+          <t>INKA PRATAMA, CV</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>7505</t>
+          <t>7501</t>
         </is>
       </c>
       <c r="I63" t="n">
-        <v>53.65853658536586</v>
+        <v>76.47058823529412</v>
       </c>
       <c r="J63" t="n">
         <v>100</v>
       </c>
       <c r="K63" t="inlineStr"/>
       <c r="L63" t="n">
-        <v>60.05046257359125</v>
+        <v>80.74866310160428</v>
       </c>
       <c r="M63" t="inlineStr">
         <is>
@@ -3834,41 +3834,41 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>MAHARANI PERSADA KONSTRUKSI, PT</t>
+          <t>MOTIKACI FAMILY GROUP, CV</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>7504</t>
+          <t>7505</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>JALAN PROF. DR. ALOE SABOE</t>
+          <t>Dusun Pasar Lama, Desa Moluo, Kecamatan Kwandang, Kabupaten Gorontalo Utara.</t>
         </is>
       </c>
       <c r="F64" t="n">
-        <v>1481</v>
+        <v>1597</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>RISKY MAHARANI ENERGI, PT</t>
+          <t>TIRTA TARUNA, CV</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>7504</t>
+          <t>7505</t>
         </is>
       </c>
       <c r="I64" t="n">
-        <v>60.71428571428572</v>
+        <v>53.65853658536586</v>
       </c>
       <c r="J64" t="n">
         <v>100</v>
       </c>
       <c r="K64" t="inlineStr"/>
       <c r="L64" t="n">
-        <v>65.20408163265307</v>
+        <v>60.05046257359125</v>
       </c>
       <c r="M64" t="inlineStr">
         <is>
@@ -3887,47 +3887,45 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>RARA BERKAH, CV</t>
+          <t>MAHARANI PERSADA KONSTRUKSI, PT</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>7571</t>
+          <t>7504</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Jalan Kancil</t>
+          <t>JALAN PROF. DR. ALOE SABOE</t>
         </is>
       </c>
       <c r="F65" t="n">
-        <v>158</v>
+        <v>1481</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>RARA BERKAH, CV</t>
+          <t>RISKY MAHARANI ENERGI, PT</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>7571</t>
+          <t>7504</t>
         </is>
       </c>
       <c r="I65" t="n">
-        <v>100</v>
+        <v>60.71428571428572</v>
       </c>
       <c r="J65" t="n">
         <v>100</v>
       </c>
-      <c r="K65" t="n">
-        <v>85.71428571428572</v>
-      </c>
+      <c r="K65" t="inlineStr"/>
       <c r="L65" t="n">
-        <v>94.47004608294931</v>
+        <v>65.20408163265307</v>
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>DROP</t>
+          <t>INSERT</t>
         </is>
       </c>
     </row>
@@ -3942,30 +3940,30 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>ALL AHAD, CV</t>
+          <t>RARA BERKAH, CV</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>7502</t>
+          <t>7571</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Jalan husin DJ Rahman</t>
+          <t>Jalan Kancil</t>
         </is>
       </c>
       <c r="F66" t="n">
-        <v>58</v>
+        <v>158</v>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>ALL AHAD, CV</t>
+          <t>RARA BERKAH, CV</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>7502</t>
+          <t>7571</t>
         </is>
       </c>
       <c r="I66" t="n">
@@ -3975,10 +3973,10 @@
         <v>100</v>
       </c>
       <c r="K66" t="n">
-        <v>92.30769230769231</v>
+        <v>85.71428571428572</v>
       </c>
       <c r="L66" t="n">
-        <v>95.63409563409563</v>
+        <v>94.47004608294931</v>
       </c>
       <c r="M66" t="inlineStr">
         <is>
@@ -3997,47 +3995,47 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>SANUR ARA, CV</t>
+          <t>ALL AHAD, CV</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>7571</t>
+          <t>7502</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Jalan Gelatik No. 26</t>
+          <t>Jalan husin DJ Rahman</t>
         </is>
       </c>
       <c r="F67" t="n">
-        <v>146</v>
+        <v>58</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>SETIA KARYA SEJATI, CV</t>
+          <t>ALL AHAD, CV</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>7571</t>
+          <t>7502</t>
         </is>
       </c>
       <c r="I67" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="J67" t="n">
         <v>100</v>
       </c>
       <c r="K67" t="n">
-        <v>78.94736842105263</v>
+        <v>92.30769230769231</v>
       </c>
       <c r="L67" t="n">
-        <v>67.53911806543385</v>
+        <v>95.63409563409563</v>
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>INSERT</t>
+          <t>DROP</t>
         </is>
       </c>
     </row>
@@ -4052,41 +4050,43 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>PUTRA ECHAXEL, CV</t>
+          <t>SANUR ARA, CV</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>7503</t>
+          <t>7571</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Jalan Sultan Botutihe</t>
+          <t>Jalan Gelatik No. 26</t>
         </is>
       </c>
       <c r="F68" t="n">
-        <v>1264</v>
+        <v>146</v>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>EKA PUTRA, CV</t>
+          <t>SETIA KARYA SEJATI, CV</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>7503</t>
+          <t>7571</t>
         </is>
       </c>
       <c r="I68" t="n">
-        <v>73.33333333333334</v>
+        <v>40</v>
       </c>
       <c r="J68" t="n">
         <v>100</v>
       </c>
-      <c r="K68" t="inlineStr"/>
+      <c r="K68" t="n">
+        <v>78.94736842105263</v>
+      </c>
       <c r="L68" t="n">
-        <v>78.41269841269842</v>
+        <v>67.53911806543385</v>
       </c>
       <c r="M68" t="inlineStr">
         <is>
@@ -4105,43 +4105,41 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>VIJAYA KARYA UTAMA, PT</t>
+          <t>PUTRA ECHAXEL, CV</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>7571</t>
+          <t>7503</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Jl. Rusli Datau 2 No 4</t>
+          <t>Jalan Sultan Botutihe</t>
         </is>
       </c>
       <c r="F69" t="n">
-        <v>2215</v>
+        <v>1264</v>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>MITRA JAYA MULTI SARANA, CV</t>
+          <t>EKA PUTRA, CV</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>7571</t>
+          <t>7503</t>
         </is>
       </c>
       <c r="I69" t="n">
-        <v>44.89795918367348</v>
+        <v>73.33333333333334</v>
       </c>
       <c r="J69" t="n">
         <v>100</v>
       </c>
-      <c r="K69" t="n">
-        <v>92.6829268292683</v>
-      </c>
+      <c r="K69" t="inlineStr"/>
       <c r="L69" t="n">
-        <v>71.3912394225983</v>
+        <v>78.41269841269842</v>
       </c>
       <c r="M69" t="inlineStr">
         <is>
@@ -4160,41 +4158,43 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>AQIFFA JAYA MANDIRI, CV</t>
+          <t>VIJAYA KARYA UTAMA, PT</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>7504</t>
+          <t>7571</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Dusun Lamahu Desa Sipatana</t>
+          <t>Jl. Rusli Datau 2 No 4</t>
         </is>
       </c>
       <c r="F70" t="n">
-        <v>1347</v>
+        <v>2215</v>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>JAYA MANDIRI PERSADA, CV</t>
+          <t>MITRA JAYA MULTI SARANA, CV</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>7504</t>
+          <t>7571</t>
         </is>
       </c>
       <c r="I70" t="n">
-        <v>68.08510638297872</v>
+        <v>44.89795918367348</v>
       </c>
       <c r="J70" t="n">
         <v>100</v>
       </c>
-      <c r="K70" t="inlineStr"/>
+      <c r="K70" t="n">
+        <v>92.6829268292683</v>
+      </c>
       <c r="L70" t="n">
-        <v>72.81323877068559</v>
+        <v>71.3912394225983</v>
       </c>
       <c r="M70" t="inlineStr">
         <is>
@@ -4213,7 +4213,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>HARMONIS PERKASAINDAH POHUWATO, PT</t>
+          <t>AQIFFA JAYA MANDIRI, CV</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -4223,15 +4223,15 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Jl. Pelabuhan</t>
+          <t>Dusun Lamahu Desa Sipatana</t>
         </is>
       </c>
       <c r="F71" t="n">
-        <v>100</v>
+        <v>1347</v>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>HARMONIS PERKASAINDAH POHUWATO, PT</t>
+          <t>JAYA MANDIRI PERSADA, CV</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -4240,20 +4240,18 @@
         </is>
       </c>
       <c r="I71" t="n">
-        <v>100</v>
+        <v>68.08510638297872</v>
       </c>
       <c r="J71" t="n">
         <v>100</v>
       </c>
-      <c r="K71" t="n">
-        <v>96</v>
-      </c>
+      <c r="K71" t="inlineStr"/>
       <c r="L71" t="n">
-        <v>98.98039215686275</v>
+        <v>72.81323877068559</v>
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t>DROP</t>
+          <t>INSERT</t>
         </is>
       </c>
     </row>
@@ -4268,7 +4266,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>EKA PUTRA, CV</t>
+          <t>HARMONIS PERKASAINDAH POHUWATO, PT</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -4278,15 +4276,15 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Jalan Gagak, depan RM ASTA 6000, Desa Marisa Selatan, Kecamatan Marisa, Kabupaten Pohuwato</t>
+          <t>Jl. Pelabuhan</t>
         </is>
       </c>
       <c r="F72" t="n">
-        <v>1419</v>
+        <v>100</v>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>LOMAYA PUTRA, CV</t>
+          <t>HARMONIS PERKASAINDAH POHUWATO, PT</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -4295,18 +4293,20 @@
         </is>
       </c>
       <c r="I72" t="n">
-        <v>75.86206896551724</v>
+        <v>100</v>
       </c>
       <c r="J72" t="n">
         <v>100</v>
       </c>
-      <c r="K72" t="inlineStr"/>
+      <c r="K72" t="n">
+        <v>96</v>
+      </c>
       <c r="L72" t="n">
-        <v>81.54158215010142</v>
+        <v>98.98039215686275</v>
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>INSERT</t>
+          <t>DROP</t>
         </is>
       </c>
     </row>
@@ -4321,43 +4321,41 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>TRI SANDI YUDHA, PT</t>
+          <t>EKA PUTRA, CV</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>7571</t>
+          <t>7504</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Jalan Jakarta, Kompleks Perum Griya Wiyan Lestari Blok D Nomor 1</t>
+          <t>Jalan Gagak, depan RM ASTA 6000, Desa Marisa Selatan, Kecamatan Marisa, Kabupaten Pohuwato</t>
         </is>
       </c>
       <c r="F73" t="n">
-        <v>119</v>
+        <v>1419</v>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>TRI SANDI YUDHA, PT</t>
+          <t>LOMAYA PUTRA, CV</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>7571</t>
+          <t>7504</t>
         </is>
       </c>
       <c r="I73" t="n">
-        <v>100</v>
+        <v>75.86206896551724</v>
       </c>
       <c r="J73" t="n">
         <v>100</v>
       </c>
-      <c r="K73" t="n">
-        <v>62.5</v>
-      </c>
+      <c r="K73" t="inlineStr"/>
       <c r="L73" t="n">
-        <v>72.41379310344827</v>
+        <v>81.54158215010142</v>
       </c>
       <c r="M73" t="inlineStr">
         <is>
@@ -4376,41 +4374,43 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>ARUMI, CV</t>
+          <t>TRI SANDI YUDHA, PT</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>7501</t>
+          <t>7571</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>JALAN SAMRATULANGI DUSUN I TENGAH, DESA YOSONEGORO, KECAMATAN LIMBOTO BARAT, KABUPATEN GORONTALO</t>
+          <t>Jalan Jakarta, Kompleks Perum Griya Wiyan Lestari Blok D Nomor 1</t>
         </is>
       </c>
       <c r="F74" t="n">
-        <v>265</v>
+        <v>119</v>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>ARSA, CV</t>
+          <t>TRI SANDI YUDHA, PT</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>7501</t>
+          <t>7571</t>
         </is>
       </c>
       <c r="I74" t="n">
-        <v>70.58823529411764</v>
+        <v>100</v>
       </c>
       <c r="J74" t="n">
         <v>100</v>
       </c>
-      <c r="K74" t="inlineStr"/>
+      <c r="K74" t="n">
+        <v>62.5</v>
+      </c>
       <c r="L74" t="n">
-        <v>79.63800904977376</v>
+        <v>72.41379310344827</v>
       </c>
       <c r="M74" t="inlineStr">
         <is>
@@ -4429,7 +4429,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>DHARMA BAKTI, CV</t>
+          <t>ARUMI, CV</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -4439,15 +4439,15 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>JL. RAYA LIMBOTO NO. 9</t>
+          <t>JALAN SAMRATULANGI DUSUN I TENGAH, DESA YOSONEGORO, KECAMATAN LIMBOTO BARAT, KABUPATEN GORONTALO</t>
         </is>
       </c>
       <c r="F75" t="n">
-        <v>421</v>
+        <v>265</v>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>RAHMAT ABADI, CV</t>
+          <t>ARSA, CV</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
@@ -4456,14 +4456,14 @@
         </is>
       </c>
       <c r="I75" t="n">
-        <v>68.75</v>
+        <v>70.58823529411764</v>
       </c>
       <c r="J75" t="n">
         <v>100</v>
       </c>
       <c r="K75" t="inlineStr"/>
       <c r="L75" t="n">
-        <v>75</v>
+        <v>79.63800904977376</v>
       </c>
       <c r="M75" t="inlineStr">
         <is>
@@ -4482,41 +4482,41 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>GOMINA PERMAI INDAH, CV</t>
+          <t>DHARMA BAKTI, CV</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>7503</t>
+          <t>7501</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Jalan Nani Wartabone</t>
+          <t>JL. RAYA LIMBOTO NO. 9</t>
         </is>
       </c>
       <c r="F76" t="n">
-        <v>1151</v>
+        <v>421</v>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>GLORIA INDAH, CV</t>
+          <t>RAHMAT ABADI, CV</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>7503</t>
+          <t>7501</t>
         </is>
       </c>
       <c r="I76" t="n">
-        <v>71.7948717948718</v>
+        <v>68.75</v>
       </c>
       <c r="J76" t="n">
         <v>100</v>
       </c>
       <c r="K76" t="inlineStr"/>
       <c r="L76" t="n">
-        <v>75.97340930674264</v>
+        <v>75</v>
       </c>
       <c r="M76" t="inlineStr">
         <is>
@@ -4535,43 +4535,45 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>ALIF SATYA PERKASA, PT</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr"/>
+          <t>GOMINA PERMAI INDAH, CV</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>7503</t>
+        </is>
+      </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>DESA TINELO</t>
+          <t>Jalan Nani Wartabone</t>
         </is>
       </c>
       <c r="F77" t="n">
-        <v>509</v>
+        <v>1151</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>ALIF SETYA PERKASA, PT</t>
+          <t>GLORIA INDAH, CV</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>7502</t>
+          <t>7503</t>
         </is>
       </c>
       <c r="I77" t="n">
-        <v>95.45454545454545</v>
+        <v>71.7948717948718</v>
       </c>
       <c r="J77" t="n">
-        <v>0</v>
-      </c>
-      <c r="K77" t="n">
-        <v>100</v>
-      </c>
+        <v>100</v>
+      </c>
+      <c r="K77" t="inlineStr"/>
       <c r="L77" t="n">
-        <v>96.96969696969697</v>
+        <v>75.97340930674264</v>
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t>DROP</t>
+          <t>INSERT</t>
         </is>
       </c>
     </row>
@@ -4586,45 +4588,43 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>MADINA MULTI KREASI, CV</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr">
-        <is>
-          <t>7501</t>
-        </is>
-      </c>
+          <t>ALIF SATYA PERKASA, PT</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr"/>
       <c r="E78" t="inlineStr">
         <is>
-          <t>JALAN JARWADI LINGKUNGAN I</t>
+          <t>DESA TINELO</t>
         </is>
       </c>
       <c r="F78" t="n">
-        <v>444</v>
+        <v>509</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>SEMANGAT KARYA, CV</t>
+          <t>ALIF SETYA PERKASA, PT</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>7501</t>
+          <t>7502</t>
         </is>
       </c>
       <c r="I78" t="n">
-        <v>63.41463414634146</v>
+        <v>95.45454545454545</v>
       </c>
       <c r="J78" t="n">
-        <v>100</v>
-      </c>
-      <c r="K78" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="K78" t="n">
+        <v>100</v>
+      </c>
       <c r="L78" t="n">
-        <v>68.83468834688347</v>
+        <v>96.96969696969697</v>
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t>INSERT</t>
+          <t>DROP</t>
         </is>
       </c>
     </row>
@@ -4639,45 +4639,43 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>SELTA LESTARI, CV</t>
-        </is>
-      </c>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>7504</t>
-        </is>
-      </c>
+          <t>ALIF SATYA PERKASA, PT</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr"/>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Dusun Teratai</t>
+          <t>DESA TINELO</t>
         </is>
       </c>
       <c r="F79" t="n">
-        <v>1434</v>
+        <v>509</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>SINAR LESTARI, CV</t>
+          <t>ALIF SETYA PERKASA, PT</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>7504</t>
+          <t>7502</t>
         </is>
       </c>
       <c r="I79" t="n">
-        <v>82.35294117647058</v>
+        <v>95.45454545454545</v>
       </c>
       <c r="J79" t="n">
-        <v>100</v>
-      </c>
-      <c r="K79" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="K79" t="n">
+        <v>100</v>
+      </c>
       <c r="L79" t="n">
-        <v>85.71428571428571</v>
+        <v>96.96969696969697</v>
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>INSERT</t>
+          <t>DROP</t>
         </is>
       </c>
     </row>
@@ -4692,47 +4690,45 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>GARUDA SAKTI, CV</t>
+          <t>MADINA MULTI KREASI, CV</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>7571</t>
+          <t>7501</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>JALAN MATOLODULA</t>
+          <t>JALAN JARWADI LINGKUNGAN I</t>
         </is>
       </c>
       <c r="F80" t="n">
-        <v>2047</v>
+        <v>444</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>GARUDA SAKTI, CV</t>
+          <t>SEMANGAT KARYA, CV</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>7571</t>
+          <t>7501</t>
         </is>
       </c>
       <c r="I80" t="n">
-        <v>100</v>
+        <v>63.41463414634146</v>
       </c>
       <c r="J80" t="n">
         <v>100</v>
       </c>
-      <c r="K80" t="n">
-        <v>89.65517241379311</v>
-      </c>
+      <c r="K80" t="inlineStr"/>
       <c r="L80" t="n">
-        <v>95.40229885057471</v>
+        <v>68.83468834688347</v>
       </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t>DROP</t>
+          <t>INSERT</t>
         </is>
       </c>
     </row>
@@ -4747,41 +4743,41 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>TULUS RAJAWALI GORONTALO, PT</t>
+          <t>SELTA LESTARI, CV</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>7503</t>
+          <t>7504</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>DESA TOTO SELATAN</t>
+          <t>Dusun Teratai</t>
         </is>
       </c>
       <c r="F81" t="n">
-        <v>1136</v>
+        <v>1434</v>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>KURNIA LOGISTIK PRATAMA, PT</t>
+          <t>SINAR LESTARI, CV</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>7503</t>
+          <t>7504</t>
         </is>
       </c>
       <c r="I81" t="n">
-        <v>47.27272727272728</v>
+        <v>82.35294117647058</v>
       </c>
       <c r="J81" t="n">
         <v>100</v>
       </c>
       <c r="K81" t="inlineStr"/>
       <c r="L81" t="n">
-        <v>53.86363636363637</v>
+        <v>85.71428571428571</v>
       </c>
       <c r="M81" t="inlineStr">
         <is>
@@ -4800,45 +4796,47 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>SINAR BATU ALAM, CV</t>
+          <t>GARUDA SAKTI, CV</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>7501</t>
+          <t>7571</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Jl. JENDRAL SUDIRMAN</t>
+          <t>JALAN MATOLODULA</t>
         </is>
       </c>
       <c r="F82" t="n">
-        <v>246</v>
+        <v>2047</v>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>SINAR ALINKO, CV</t>
+          <t>GARUDA SAKTI, CV</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>7501</t>
+          <t>7571</t>
         </is>
       </c>
       <c r="I82" t="n">
-        <v>68.57142857142857</v>
+        <v>100</v>
       </c>
       <c r="J82" t="n">
         <v>100</v>
       </c>
-      <c r="K82" t="inlineStr"/>
+      <c r="K82" t="n">
+        <v>89.65517241379311</v>
+      </c>
       <c r="L82" t="n">
-        <v>74.03726708074534</v>
+        <v>95.40229885057471</v>
       </c>
       <c r="M82" t="inlineStr">
         <is>
-          <t>INSERT</t>
+          <t>DROP</t>
         </is>
       </c>
     </row>
@@ -4853,47 +4851,45 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>PUTRA DEZA, CV</t>
+          <t>TULUS RAJAWALI GORONTALO, PT</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>7501</t>
+          <t>7503</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>DUSUN MUARA</t>
+          <t>DESA TOTO SELATAN</t>
         </is>
       </c>
       <c r="F83" t="n">
-        <v>34</v>
+        <v>1136</v>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>PUTRA DEZA, CV</t>
+          <t>KURNIA LOGISTIK PRATAMA, PT</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>7501</t>
+          <t>7503</t>
         </is>
       </c>
       <c r="I83" t="n">
-        <v>100</v>
+        <v>47.27272727272728</v>
       </c>
       <c r="J83" t="n">
         <v>100</v>
       </c>
-      <c r="K83" t="n">
-        <v>90</v>
-      </c>
+      <c r="K83" t="inlineStr"/>
       <c r="L83" t="n">
-        <v>96.20689655172414</v>
+        <v>53.86363636363637</v>
       </c>
       <c r="M83" t="inlineStr">
         <is>
-          <t>DROP</t>
+          <t>INSERT</t>
         </is>
       </c>
     </row>
@@ -4908,41 +4904,41 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>ABADI JAYA BERSAMA NEW, CV</t>
+          <t>SINAR BATU ALAM, CV</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>7504</t>
+          <t>7501</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>DESA BUNUYO KECAMATAN PAGUAT</t>
+          <t>Jl. JENDRAL SUDIRMAN</t>
         </is>
       </c>
       <c r="F84" t="n">
-        <v>1392</v>
+        <v>246</v>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>CITRA ABDI KARYA, CV</t>
+          <t>SINAR ALINKO, CV</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>7504</t>
+          <t>7501</t>
         </is>
       </c>
       <c r="I84" t="n">
-        <v>65.21739130434783</v>
+        <v>68.57142857142857</v>
       </c>
       <c r="J84" t="n">
         <v>100</v>
       </c>
       <c r="K84" t="inlineStr"/>
       <c r="L84" t="n">
-        <v>69.85507246376811</v>
+        <v>74.03726708074534</v>
       </c>
       <c r="M84" t="inlineStr">
         <is>
@@ -4961,7 +4957,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>ARMADAN JAYA, CV</t>
+          <t>PUTRA DEZA, CV</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -4971,15 +4967,15 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Jalan Hasan Dangkua Lingkungan I</t>
+          <t>DUSUN MUARA</t>
         </is>
       </c>
       <c r="F85" t="n">
-        <v>275</v>
+        <v>34</v>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>CAHAYA AGRO KARYA, CV</t>
+          <t>PUTRA DEZA, CV</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
@@ -4988,18 +4984,20 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>64.86486486486487</v>
+        <v>100</v>
       </c>
       <c r="J85" t="n">
         <v>100</v>
       </c>
-      <c r="K85" t="inlineStr"/>
+      <c r="K85" t="n">
+        <v>90</v>
+      </c>
       <c r="L85" t="n">
-        <v>71.8918918918919</v>
+        <v>96.20689655172414</v>
       </c>
       <c r="M85" t="inlineStr">
         <is>
-          <t>INSERT</t>
+          <t>DROP</t>
         </is>
       </c>
     </row>
@@ -5014,43 +5012,41 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>SURYA SINTESIA, CV</t>
+          <t>ABADI JAYA BERSAMA NEW, CV</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>7571</t>
+          <t>7504</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>JALAN PADANG PERUMAHAN GRAHA 42 BLOK E NO.3</t>
+          <t>DESA BUNUYO KECAMATAN PAGUAT</t>
         </is>
       </c>
       <c r="F86" t="n">
-        <v>2214</v>
+        <v>1392</v>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>SURYA SINTESIA, CV</t>
+          <t>CITRA ABDI KARYA, CV</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>7571</t>
+          <t>7504</t>
         </is>
       </c>
       <c r="I86" t="n">
-        <v>100</v>
+        <v>65.21739130434783</v>
       </c>
       <c r="J86" t="n">
         <v>100</v>
       </c>
-      <c r="K86" t="n">
-        <v>50.84745762711864</v>
-      </c>
+      <c r="K86" t="inlineStr"/>
       <c r="L86" t="n">
-        <v>67.48370273794004</v>
+        <v>69.85507246376811</v>
       </c>
       <c r="M86" t="inlineStr">
         <is>
@@ -5069,41 +5065,41 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>SENCIKA INDAH, CV</t>
+          <t>ARMADAN JAYA, CV</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>7504</t>
+          <t>7501</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Jln. Pelabuhan Marisa</t>
+          <t>Jalan Hasan Dangkua Lingkungan I</t>
         </is>
       </c>
       <c r="F87" t="n">
-        <v>1442</v>
+        <v>275</v>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>NUSA INDAH, CV</t>
+          <t>CAHAYA AGRO KARYA, CV</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>7504</t>
+          <t>7501</t>
         </is>
       </c>
       <c r="I87" t="n">
-        <v>77.41935483870968</v>
+        <v>64.86486486486487</v>
       </c>
       <c r="J87" t="n">
         <v>100</v>
       </c>
       <c r="K87" t="inlineStr"/>
       <c r="L87" t="n">
-        <v>81.72043010752688</v>
+        <v>71.8918918918919</v>
       </c>
       <c r="M87" t="inlineStr">
         <is>
@@ -5122,7 +5118,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>ANDARA ARTHA KONSTRUKSI, PT</t>
+          <t>SURYA SINTESIA, CV</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -5132,15 +5128,15 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>JALAN CUT NYAK DIEN</t>
+          <t>JALAN PADANG PERUMAHAN GRAHA 42 BLOK E NO.3</t>
         </is>
       </c>
       <c r="F88" t="n">
-        <v>2194</v>
+        <v>2214</v>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>ANDARA ARTHA KONSTRUKSI, PT</t>
+          <t>SURYA SINTESIA, CV</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
@@ -5155,14 +5151,14 @@
         <v>100</v>
       </c>
       <c r="K88" t="n">
-        <v>91.42857142857143</v>
+        <v>50.84745762711864</v>
       </c>
       <c r="L88" t="n">
-        <v>96.74285714285713</v>
+        <v>67.48370273794004</v>
       </c>
       <c r="M88" t="inlineStr">
         <is>
-          <t>DROP</t>
+          <t>INSERT</t>
         </is>
       </c>
     </row>
@@ -5177,41 +5173,41 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>SINAR PUTRI PRATAMA, CV</t>
+          <t>SENCIKA INDAH, CV</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>7501</t>
+          <t>7504</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Jalan PGRI</t>
+          <t>Jln. Pelabuhan Marisa</t>
         </is>
       </c>
       <c r="F89" t="n">
-        <v>375</v>
+        <v>1442</v>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>SINAR PURNAMA, CV</t>
+          <t>NUSA INDAH, CV</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>7501</t>
+          <t>7504</t>
         </is>
       </c>
       <c r="I89" t="n">
-        <v>75</v>
+        <v>77.41935483870968</v>
       </c>
       <c r="J89" t="n">
         <v>100</v>
       </c>
       <c r="K89" t="inlineStr"/>
       <c r="L89" t="n">
-        <v>78.70370370370371</v>
+        <v>81.72043010752688</v>
       </c>
       <c r="M89" t="inlineStr">
         <is>
@@ -5230,45 +5226,47 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>BAYOORS, CV</t>
+          <t>ANDARA ARTHA KONSTRUKSI, PT</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>7503</t>
+          <t>7571</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Jl. -</t>
+          <t>JALAN CUT NYAK DIEN</t>
         </is>
       </c>
       <c r="F90" t="n">
-        <v>1139</v>
+        <v>2194</v>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>CITOS, CV</t>
+          <t>ANDARA ARTHA KONSTRUKSI, PT</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>7503</t>
+          <t>7571</t>
         </is>
       </c>
       <c r="I90" t="n">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="J90" t="n">
         <v>100</v>
       </c>
-      <c r="K90" t="inlineStr"/>
+      <c r="K90" t="n">
+        <v>91.42857142857143</v>
+      </c>
       <c r="L90" t="n">
-        <v>70.66666666666667</v>
+        <v>96.74285714285713</v>
       </c>
       <c r="M90" t="inlineStr">
         <is>
-          <t>INSERT</t>
+          <t>DROP</t>
         </is>
       </c>
     </row>
@@ -5283,7 +5281,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>KARYA JAYA BERSAMA, CV</t>
+          <t>SINAR PUTRI PRATAMA, CV</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -5293,15 +5291,15 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Dusun Motolohu</t>
+          <t>Jalan PGRI</t>
         </is>
       </c>
       <c r="F91" t="n">
-        <v>227</v>
+        <v>375</v>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>KARYA BERSAMA, CV</t>
+          <t>SINAR PURNAMA, CV</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
@@ -5310,16 +5308,14 @@
         </is>
       </c>
       <c r="I91" t="n">
-        <v>87.17948717948718</v>
+        <v>75</v>
       </c>
       <c r="J91" t="n">
         <v>100</v>
       </c>
-      <c r="K91" t="n">
-        <v>27.45098039215686</v>
-      </c>
+      <c r="K91" t="inlineStr"/>
       <c r="L91" t="n">
-        <v>67.55656108597285</v>
+        <v>78.70370370370371</v>
       </c>
       <c r="M91" t="inlineStr">
         <is>
@@ -5338,43 +5334,41 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>ALYA BERKAH, CV</t>
+          <t>BAYOORS, CV</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>7571</t>
+          <t>7503</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Jalan Kancil</t>
+          <t>Jl. -</t>
         </is>
       </c>
       <c r="F92" t="n">
-        <v>158</v>
+        <v>1139</v>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>RARA BERKAH, CV</t>
+          <t>CITOS, CV</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>7571</t>
+          <t>7503</t>
         </is>
       </c>
       <c r="I92" t="n">
-        <v>66.66666666666667</v>
+        <v>60</v>
       </c>
       <c r="J92" t="n">
         <v>100</v>
       </c>
-      <c r="K92" t="n">
-        <v>85.71428571428572</v>
-      </c>
+      <c r="K92" t="inlineStr"/>
       <c r="L92" t="n">
-        <v>78.34101382488478</v>
+        <v>70.66666666666667</v>
       </c>
       <c r="M92" t="inlineStr">
         <is>
@@ -5393,7 +5387,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>INDAH RAHAYU, CV</t>
+          <t>KARYA JAYA BERSAMA, CV</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -5403,15 +5397,15 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>JALAN JENDERAL SUDIRMAN NOMOR 28</t>
+          <t>Dusun Motolohu</t>
         </is>
       </c>
       <c r="F93" t="n">
-        <v>291</v>
+        <v>227</v>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>INDAH KERAMIK, CV</t>
+          <t>KARYA BERSAMA, CV</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
@@ -5420,14 +5414,16 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>72.72727272727273</v>
+        <v>87.17948717948718</v>
       </c>
       <c r="J93" t="n">
         <v>100</v>
       </c>
-      <c r="K93" t="inlineStr"/>
+      <c r="K93" t="n">
+        <v>27.45098039215686</v>
+      </c>
       <c r="L93" t="n">
-        <v>78.18181818181819</v>
+        <v>67.55656108597285</v>
       </c>
       <c r="M93" t="inlineStr">
         <is>
@@ -5446,41 +5442,41 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>NURUL YAKIN, CV</t>
+          <t>INDAH RAHAYU, CV</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>7504</t>
+          <t>7501</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Jln. Sultan Amai</t>
+          <t>JALAN JENDERAL SUDIRMAN NOMOR 28</t>
         </is>
       </c>
       <c r="F94" t="n">
-        <v>1431</v>
+        <v>291</v>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>RIDWAN, CV</t>
+          <t>INDAH KERAMIK, CV</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>7504</t>
+          <t>7501</t>
         </is>
       </c>
       <c r="I94" t="n">
-        <v>56.00000000000001</v>
+        <v>72.72727272727273</v>
       </c>
       <c r="J94" t="n">
         <v>100</v>
       </c>
       <c r="K94" t="inlineStr"/>
       <c r="L94" t="n">
-        <v>65.26315789473684</v>
+        <v>78.18181818181819</v>
       </c>
       <c r="M94" t="inlineStr">
         <is>
@@ -5499,41 +5495,41 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>WAHYU, CV</t>
+          <t>NURUL YAKIN, CV</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>7503</t>
+          <t>7504</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Jl. Kesehatan, Desa Toto Utara</t>
+          <t>Jln. Sultan Amai</t>
         </is>
       </c>
       <c r="F95" t="n">
-        <v>1160</v>
+        <v>1431</v>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>JDS RAYA, CV</t>
+          <t>RIDWAN, CV</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>7503</t>
+          <t>7504</t>
         </is>
       </c>
       <c r="I95" t="n">
-        <v>57.14285714285714</v>
+        <v>56.00000000000001</v>
       </c>
       <c r="J95" t="n">
         <v>100</v>
       </c>
       <c r="K95" t="inlineStr"/>
       <c r="L95" t="n">
-        <v>70.32967032967032</v>
+        <v>65.26315789473684</v>
       </c>
       <c r="M95" t="inlineStr">
         <is>
@@ -5552,47 +5548,45 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>SUNGAI BONE GORONTALO, CV</t>
+          <t>WAHYU, CV</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>7571</t>
+          <t>7503</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>JALAN PALMA</t>
+          <t>Jl. Kesehatan, Desa Toto Utara</t>
         </is>
       </c>
       <c r="F96" t="n">
-        <v>2098</v>
+        <v>1160</v>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>SUNGAI BONE GORONTALO, CV</t>
+          <t>JDS RAYA, CV</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>7571</t>
+          <t>7503</t>
         </is>
       </c>
       <c r="I96" t="n">
-        <v>100</v>
+        <v>57.14285714285714</v>
       </c>
       <c r="J96" t="n">
         <v>100</v>
       </c>
-      <c r="K96" t="n">
-        <v>44.99999999999999</v>
-      </c>
+      <c r="K96" t="inlineStr"/>
       <c r="L96" t="n">
-        <v>84.875</v>
+        <v>70.32967032967032</v>
       </c>
       <c r="M96" t="inlineStr">
         <is>
-          <t>DROP</t>
+          <t>INSERT</t>
         </is>
       </c>
     </row>
@@ -5607,45 +5601,47 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>CAHAYA BULAN, CV</t>
+          <t>SUNGAI BONE GORONTALO, CV</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>7501</t>
+          <t>7571</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Dusun Lamahu</t>
+          <t>JALAN PALMA</t>
         </is>
       </c>
       <c r="F97" t="n">
-        <v>414</v>
+        <v>2098</v>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>CAHAYA AGUNG, CV</t>
+          <t>SUNGAI BONE GORONTALO, CV</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>7501</t>
+          <t>7571</t>
         </is>
       </c>
       <c r="I97" t="n">
-        <v>81.25</v>
+        <v>100</v>
       </c>
       <c r="J97" t="n">
         <v>100</v>
       </c>
-      <c r="K97" t="inlineStr"/>
+      <c r="K97" t="n">
+        <v>44.99999999999999</v>
+      </c>
       <c r="L97" t="n">
-        <v>85</v>
+        <v>84.875</v>
       </c>
       <c r="M97" t="inlineStr">
         <is>
-          <t>INSERT</t>
+          <t>DROP</t>
         </is>
       </c>
     </row>
@@ -5660,47 +5656,45 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>ALLIESSAN, PT</t>
+          <t>CAHAYA BULAN, CV</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>7571</t>
+          <t>7501</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>JL. SULTAN HASANUDDIN</t>
+          <t>Dusun Lamahu</t>
         </is>
       </c>
       <c r="F98" t="n">
-        <v>2240</v>
+        <v>414</v>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>ALLIESSAN, PT</t>
+          <t>CAHAYA AGUNG, CV</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>7571</t>
+          <t>7501</t>
         </is>
       </c>
       <c r="I98" t="n">
-        <v>100</v>
+        <v>81.25</v>
       </c>
       <c r="J98" t="n">
         <v>100</v>
       </c>
-      <c r="K98" t="n">
-        <v>95</v>
-      </c>
+      <c r="K98" t="inlineStr"/>
       <c r="L98" t="n">
-        <v>97.23684210526316</v>
+        <v>85</v>
       </c>
       <c r="M98" t="inlineStr">
         <is>
-          <t>DROP</t>
+          <t>INSERT</t>
         </is>
       </c>
     </row>
@@ -5715,7 +5709,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>RAHLIN AULIA MANDIRI, PT</t>
+          <t>ALLIESSAN, PT</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -5725,15 +5719,15 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Jalan Beringin</t>
+          <t>JL. SULTAN HASANUDDIN</t>
         </is>
       </c>
       <c r="F99" t="n">
-        <v>1683</v>
+        <v>2240</v>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>RAHLIN AULIA MANDIRI, PT</t>
+          <t>ALLIESSAN, PT</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
@@ -5748,10 +5742,10 @@
         <v>100</v>
       </c>
       <c r="K99" t="n">
-        <v>50.90909090909091</v>
+        <v>95</v>
       </c>
       <c r="L99" t="n">
-        <v>83.63636363636364</v>
+        <v>97.23684210526316</v>
       </c>
       <c r="M99" t="inlineStr">
         <is>
@@ -5770,45 +5764,47 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>ZIITEK, CV</t>
+          <t>RAHLIN AULIA MANDIRI, PT</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>7503</t>
+          <t>7571</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Desa Toto Utara, Kecamatan Tilongkabila, Kabupaten Bone Bolango</t>
+          <t>Jalan Beringin</t>
         </is>
       </c>
       <c r="F100" t="n">
-        <v>1208</v>
+        <v>1683</v>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>SPEKTEK, CV</t>
+          <t>RAHLIN AULIA MANDIRI, PT</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>7503</t>
+          <t>7571</t>
         </is>
       </c>
       <c r="I100" t="n">
-        <v>66.66666666666667</v>
+        <v>100</v>
       </c>
       <c r="J100" t="n">
         <v>100</v>
       </c>
-      <c r="K100" t="inlineStr"/>
+      <c r="K100" t="n">
+        <v>50.90909090909091</v>
+      </c>
       <c r="L100" t="n">
-        <v>76.19047619047619</v>
+        <v>83.63636363636364</v>
       </c>
       <c r="M100" t="inlineStr">
         <is>
-          <t>INSERT</t>
+          <t>DROP</t>
         </is>
       </c>
     </row>
@@ -5823,41 +5819,41 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>USAHA SEJAHTERA, CV</t>
+          <t>ZIITEK, CV</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>7504</t>
+          <t>7503</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Jl. Pelabuhan</t>
+          <t>Desa Toto Utara, Kecamatan Tilongkabila, Kabupaten Bone Bolango</t>
         </is>
       </c>
       <c r="F101" t="n">
-        <v>1404</v>
+        <v>1208</v>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>BRESCIA SEJAHTERA SELATAN, PT</t>
+          <t>SPEKTEK, CV</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>7504</t>
+          <t>7503</t>
         </is>
       </c>
       <c r="I101" t="n">
-        <v>62.5</v>
+        <v>66.66666666666667</v>
       </c>
       <c r="J101" t="n">
         <v>100</v>
       </c>
       <c r="K101" t="inlineStr"/>
       <c r="L101" t="n">
-        <v>69.02173913043478</v>
+        <v>76.19047619047619</v>
       </c>
       <c r="M101" t="inlineStr">
         <is>
@@ -5876,41 +5872,41 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>TRIANA, CV</t>
+          <t>USAHA SEJAHTERA, CV</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>7501</t>
+          <t>7504</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Perum Azizah Permai Blok I Nomor 3</t>
+          <t>Jl. Pelabuhan</t>
         </is>
       </c>
       <c r="F102" t="n">
-        <v>364</v>
+        <v>1404</v>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>PRIMADONA, CV</t>
+          <t>BRESCIA SEJAHTERA SELATAN, PT</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>7501</t>
+          <t>7504</t>
         </is>
       </c>
       <c r="I102" t="n">
-        <v>78.26086956521739</v>
+        <v>62.5</v>
       </c>
       <c r="J102" t="n">
         <v>100</v>
       </c>
       <c r="K102" t="inlineStr"/>
       <c r="L102" t="n">
-        <v>84.47204968944099</v>
+        <v>69.02173913043478</v>
       </c>
       <c r="M102" t="inlineStr">
         <is>
@@ -5929,7 +5925,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>BINTANG ADZKIA, CV</t>
+          <t>TRIANA, CV</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -5939,15 +5935,15 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Jalan A. Otoluwa</t>
+          <t>Perum Azizah Permai Blok I Nomor 3</t>
         </is>
       </c>
       <c r="F103" t="n">
-        <v>263</v>
+        <v>364</v>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>ANUGERAH ABADI, CV</t>
+          <t>PRIMADONA, CV</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
@@ -5956,14 +5952,14 @@
         </is>
       </c>
       <c r="I103" t="n">
-        <v>61.11111111111111</v>
+        <v>78.26086956521739</v>
       </c>
       <c r="J103" t="n">
         <v>100</v>
       </c>
       <c r="K103" t="inlineStr"/>
       <c r="L103" t="n">
-        <v>68.18181818181819</v>
+        <v>84.47204968944099</v>
       </c>
       <c r="M103" t="inlineStr">
         <is>
@@ -5974,49 +5970,49 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>lpse</t>
+          <t>sijk</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>0</v>
+        <v>102</v>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>HADFIR PERKASA, CV</t>
+          <t>BINTANG ADZKIA, CV</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>7502</t>
+          <t>7501</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>PERUM PADENGO PERMAI 6 BLOK C NOMOR 1 TENGGELA KECAMATAN TILANGO</t>
+          <t>Jalan A. Otoluwa</t>
         </is>
       </c>
       <c r="F104" t="n">
-        <v>844</v>
+        <v>263</v>
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>DWI AULIA PERKASA, CV</t>
+          <t>ANUGERAH ABADI, CV</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>7502</t>
+          <t>7501</t>
         </is>
       </c>
       <c r="I104" t="n">
-        <v>71.7948717948718</v>
+        <v>61.11111111111111</v>
       </c>
       <c r="J104" t="n">
         <v>100</v>
       </c>
       <c r="K104" t="inlineStr"/>
       <c r="L104" t="n">
-        <v>76.92307692307692</v>
+        <v>68.18181818181819</v>
       </c>
       <c r="M104" t="inlineStr">
         <is>
@@ -6031,45 +6027,45 @@
         </is>
       </c>
       <c r="B105" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>TULUS MULIA, CV</t>
+          <t>HADFIR PERKASA, CV</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>7571</t>
+          <t>7502</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Jl. Gunung Boliohuto No 96 Rt. 003 Rw. 005 Kel. Biawu Kec. Kota Selatan</t>
+          <t>PERUM PADENGO PERMAI 6 BLOK C NOMOR 1 TENGGELA KECAMATAN TILANGO</t>
         </is>
       </c>
       <c r="F105" t="n">
-        <v>1906</v>
+        <v>844</v>
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>LIMA SATU, CV</t>
+          <t>DWI AULIA PERKASA, CV</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>7571</t>
+          <t>7502</t>
         </is>
       </c>
       <c r="I105" t="n">
-        <v>64.28571428571428</v>
+        <v>71.7948717948718</v>
       </c>
       <c r="J105" t="n">
         <v>100</v>
       </c>
       <c r="K105" t="inlineStr"/>
       <c r="L105" t="n">
-        <v>71.80451127819549</v>
+        <v>76.92307692307692</v>
       </c>
       <c r="M105" t="inlineStr">
         <is>
@@ -6084,45 +6080,45 @@
         </is>
       </c>
       <c r="B106" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>DWI SAMA, CV</t>
+          <t>TULUS MULIA, CV</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>7504</t>
+          <t>7571</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>DESA TALANGO KECAMATAN KABILA</t>
+          <t>Jl. Gunung Boliohuto No 96 Rt. 003 Rw. 005 Kel. Biawu Kec. Kota Selatan</t>
         </is>
       </c>
       <c r="F106" t="n">
-        <v>1408</v>
+        <v>1906</v>
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>DIRAHMATI, CV</t>
+          <t>LIMA SATU, CV</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>7504</t>
+          <t>7571</t>
         </is>
       </c>
       <c r="I106" t="n">
-        <v>72</v>
+        <v>64.28571428571428</v>
       </c>
       <c r="J106" t="n">
         <v>100</v>
       </c>
       <c r="K106" t="inlineStr"/>
       <c r="L106" t="n">
-        <v>79</v>
+        <v>71.80451127819549</v>
       </c>
       <c r="M106" t="inlineStr">
         <is>
@@ -6137,47 +6133,45 @@
         </is>
       </c>
       <c r="B107" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>AZRAM MAJU BERSAMA, CV</t>
+          <t>DWI SAMA, CV</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>7571</t>
+          <t>7504</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Jln Palama Kel. Libuo Kec. Dungingi</t>
+          <t>DESA TALANGO KECAMATAN KABILA</t>
         </is>
       </c>
       <c r="F107" t="n">
-        <v>145</v>
+        <v>1408</v>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>AZRAM MAJU BERSAMA, CV</t>
+          <t>DIRAHMATI, CV</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>7571</t>
+          <t>7504</t>
         </is>
       </c>
       <c r="I107" t="n">
-        <v>100</v>
+        <v>72</v>
       </c>
       <c r="J107" t="n">
         <v>100</v>
       </c>
-      <c r="K107" t="n">
-        <v>42.30769230769231</v>
-      </c>
+      <c r="K107" t="inlineStr"/>
       <c r="L107" t="n">
-        <v>66.89785624211854</v>
+        <v>79</v>
       </c>
       <c r="M107" t="inlineStr">
         <is>
@@ -6192,34 +6186,34 @@
         </is>
       </c>
       <c r="B108" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>AMIN, CV</t>
+          <t>AZRAM MAJU BERSAMA, CV</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>7504</t>
+          <t>7571</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Jalan Naniwartabone No:144 Kel Oluhuta Kec Kabila</t>
+          <t>Jln Palama Kel. Libuo Kec. Dungingi</t>
         </is>
       </c>
       <c r="F108" t="n">
-        <v>1400</v>
+        <v>145</v>
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>AMIN, CV</t>
+          <t>AZRAM MAJU BERSAMA, CV</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>7504</t>
+          <t>7571</t>
         </is>
       </c>
       <c r="I108" t="n">
@@ -6228,13 +6222,15 @@
       <c r="J108" t="n">
         <v>100</v>
       </c>
-      <c r="K108" t="inlineStr"/>
+      <c r="K108" t="n">
+        <v>42.30769230769231</v>
+      </c>
       <c r="L108" t="n">
-        <v>100</v>
+        <v>66.89785624211854</v>
       </c>
       <c r="M108" t="inlineStr">
         <is>
-          <t>DROP</t>
+          <t>INSERT</t>
         </is>
       </c>
     </row>
@@ -6245,51 +6241,49 @@
         </is>
       </c>
       <c r="B109" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>BINTANG PALMA, CV</t>
+          <t>AMIN, CV</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>7571</t>
+          <t>7504</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Jln Palma Kel. Libuo Kec. Dungingi Kota Gorontalo</t>
+          <t>Jalan Naniwartabone No:144 Kel Oluhuta Kec Kabila</t>
         </is>
       </c>
       <c r="F109" t="n">
-        <v>1955</v>
+        <v>1400</v>
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>ADI CIPTA UTAMAI, CV</t>
+          <t>AMIN, CV</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>7571</t>
+          <t>7504</t>
         </is>
       </c>
       <c r="I109" t="n">
-        <v>59.45945945945945</v>
+        <v>100</v>
       </c>
       <c r="J109" t="n">
         <v>100</v>
       </c>
-      <c r="K109" t="n">
-        <v>55.67010309278351</v>
-      </c>
+      <c r="K109" t="inlineStr"/>
       <c r="L109" t="n">
-        <v>59.12351231938861</v>
+        <v>100</v>
       </c>
       <c r="M109" t="inlineStr">
         <is>
-          <t>INSERT</t>
+          <t>DROP</t>
         </is>
       </c>
     </row>
@@ -6300,11 +6294,11 @@
         </is>
       </c>
       <c r="B110" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>MITRA CAHAYA TANAMON, CV</t>
+          <t>BINTANG PALMA, CV</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -6314,7 +6308,7 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Jl. Membramo II Kel. Molosifat U Kec. Sipatana</t>
+          <t>Jln Palma Kel. Libuo Kec. Dungingi Kota Gorontalo</t>
         </is>
       </c>
       <c r="F110" t="n">
@@ -6331,16 +6325,16 @@
         </is>
       </c>
       <c r="I110" t="n">
-        <v>50</v>
+        <v>59.45945945945945</v>
       </c>
       <c r="J110" t="n">
         <v>100</v>
       </c>
       <c r="K110" t="n">
-        <v>68.08510638297872</v>
+        <v>55.67010309278351</v>
       </c>
       <c r="L110" t="n">
-        <v>63.94479585968948</v>
+        <v>59.12351231938861</v>
       </c>
       <c r="M110" t="inlineStr">
         <is>
@@ -6355,45 +6349,47 @@
         </is>
       </c>
       <c r="B111" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>RIZKY ADITYA PRATAMA, CV</t>
+          <t>MITRA CAHAYA TANAMON, CV</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>7504</t>
+          <t>7571</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Desa Tanah Putih Kecamatan Botupingge</t>
+          <t>Jl. Membramo II Kel. Molosifat U Kec. Sipatana</t>
         </is>
       </c>
       <c r="F111" t="n">
-        <v>1492</v>
+        <v>1955</v>
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>TITIAN PRATAMA, CV</t>
+          <t>ADI CIPTA UTAMAI, CV</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>7504</t>
+          <t>7571</t>
         </is>
       </c>
       <c r="I111" t="n">
-        <v>61.90476190476191</v>
+        <v>50</v>
       </c>
       <c r="J111" t="n">
         <v>100</v>
       </c>
-      <c r="K111" t="inlineStr"/>
+      <c r="K111" t="n">
+        <v>68.08510638297872</v>
+      </c>
       <c r="L111" t="n">
-        <v>67.34693877551021</v>
+        <v>63.94479585968948</v>
       </c>
       <c r="M111" t="inlineStr">
         <is>
@@ -6408,45 +6404,45 @@
         </is>
       </c>
       <c r="B112" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>ARITO PRATAMA, CV</t>
+          <t>RIZKY ADITYA PRATAMA, CV</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>7501</t>
+          <t>7504</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>JL. TRANS SULAWESI DESA MOLOMBULAHE KECAMATAN PAGUYAMAN</t>
+          <t>Desa Tanah Putih Kecamatan Botupingge</t>
         </is>
       </c>
       <c r="F112" t="n">
-        <v>251</v>
+        <v>1492</v>
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>ARYA PRATAMA, CV</t>
+          <t>TITIAN PRATAMA, CV</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>7501</t>
+          <t>7504</t>
         </is>
       </c>
       <c r="I112" t="n">
-        <v>84.84848484848484</v>
+        <v>61.90476190476191</v>
       </c>
       <c r="J112" t="n">
         <v>100</v>
       </c>
       <c r="K112" t="inlineStr"/>
       <c r="L112" t="n">
-        <v>87.73448773448773</v>
+        <v>67.34693877551021</v>
       </c>
       <c r="M112" t="inlineStr">
         <is>
@@ -6461,45 +6457,45 @@
         </is>
       </c>
       <c r="B113" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>ANUGERAH BERSAMA, CV</t>
+          <t>ARITO PRATAMA, CV</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>7502</t>
+          <t>7501</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Jln Basoe Bobihoe</t>
+          <t>JL. TRANS SULAWESI DESA MOLOMBULAHE KECAMATAN PAGUYAMAN</t>
         </is>
       </c>
       <c r="F113" t="n">
-        <v>828</v>
+        <v>251</v>
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>BERKAH ANUGRAH, CV</t>
+          <t>ARYA PRATAMA, CV</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>7502</t>
+          <t>7501</t>
         </is>
       </c>
       <c r="I113" t="n">
-        <v>78.94736842105263</v>
+        <v>84.84848484848484</v>
       </c>
       <c r="J113" t="n">
         <v>100</v>
       </c>
       <c r="K113" t="inlineStr"/>
       <c r="L113" t="n">
-        <v>82.45614035087719</v>
+        <v>87.73448773448773</v>
       </c>
       <c r="M113" t="inlineStr">
         <is>
@@ -6514,51 +6510,49 @@
         </is>
       </c>
       <c r="B114" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>ARVID, CV</t>
+          <t>ANUGERAH BERSAMA, CV</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>7571</t>
+          <t>7502</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Jln. Jambura</t>
+          <t>Jln Basoe Bobihoe</t>
         </is>
       </c>
       <c r="F114" t="n">
-        <v>157</v>
+        <v>828</v>
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>ARVID, CV</t>
+          <t>BERKAH ANUGRAH, CV</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>7571</t>
+          <t>7502</t>
         </is>
       </c>
       <c r="I114" t="n">
-        <v>100</v>
+        <v>78.94736842105263</v>
       </c>
       <c r="J114" t="n">
         <v>100</v>
       </c>
-      <c r="K114" t="n">
-        <v>90.90909090909091</v>
-      </c>
+      <c r="K114" t="inlineStr"/>
       <c r="L114" t="n">
-        <v>95.63636363636364</v>
+        <v>82.45614035087719</v>
       </c>
       <c r="M114" t="inlineStr">
         <is>
-          <t>DROP</t>
+          <t>INSERT</t>
         </is>
       </c>
     </row>
@@ -6569,34 +6563,34 @@
         </is>
       </c>
       <c r="B115" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>PRIMADONA, CV</t>
+          <t>ARVID, CV</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>7501</t>
+          <t>7571</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Desa Limbato Kec. Tilamuta</t>
+          <t>Jln. Jambura</t>
         </is>
       </c>
       <c r="F115" t="n">
-        <v>364</v>
+        <v>157</v>
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>PRIMADONA, CV</t>
+          <t>ARVID, CV</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>7501</t>
+          <t>7571</t>
         </is>
       </c>
       <c r="I115" t="n">
@@ -6605,9 +6599,11 @@
       <c r="J115" t="n">
         <v>100</v>
       </c>
-      <c r="K115" t="inlineStr"/>
+      <c r="K115" t="n">
+        <v>90.90909090909091</v>
+      </c>
       <c r="L115" t="n">
-        <v>100</v>
+        <v>95.63636363636364</v>
       </c>
       <c r="M115" t="inlineStr">
         <is>
@@ -6622,11 +6618,11 @@
         </is>
       </c>
       <c r="B116" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>ALL AHAD, CV</t>
+          <t>PRIMADONA, CV</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -6636,15 +6632,15 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Desa Limbato Kec. Tilamuta Kab. Boalemo</t>
+          <t>Desa Limbato Kec. Tilamuta</t>
         </is>
       </c>
       <c r="F116" t="n">
-        <v>267</v>
+        <v>364</v>
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>BAROKAH ABADI, CV</t>
+          <t>PRIMADONA, CV</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
@@ -6653,18 +6649,18 @@
         </is>
       </c>
       <c r="I116" t="n">
-        <v>62.06896551724138</v>
+        <v>100</v>
       </c>
       <c r="J116" t="n">
         <v>100</v>
       </c>
       <c r="K116" t="inlineStr"/>
       <c r="L116" t="n">
-        <v>71.55172413793103</v>
+        <v>100</v>
       </c>
       <c r="M116" t="inlineStr">
         <is>
-          <t>INSERT</t>
+          <t>DROP</t>
         </is>
       </c>
     </row>
@@ -6675,47 +6671,45 @@
         </is>
       </c>
       <c r="B117" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>SATYA HARDANA, CV</t>
+          <t>ALL AHAD, CV</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>7571</t>
+          <t>7501</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>PERUM AWARA LILUWO KEC. KOTA TENGAH</t>
+          <t>Desa Limbato Kec. Tilamuta Kab. Boalemo</t>
         </is>
       </c>
       <c r="F117" t="n">
-        <v>138</v>
+        <v>267</v>
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>SATYA HARDANA, CV</t>
+          <t>BAROKAH ABADI, CV</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>7571</t>
+          <t>7501</t>
         </is>
       </c>
       <c r="I117" t="n">
-        <v>100</v>
+        <v>62.06896551724138</v>
       </c>
       <c r="J117" t="n">
         <v>100</v>
       </c>
-      <c r="K117" t="n">
-        <v>53.84615384615385</v>
-      </c>
+      <c r="K117" t="inlineStr"/>
       <c r="L117" t="n">
-        <v>71.15384615384616</v>
+        <v>71.55172413793103</v>
       </c>
       <c r="M117" t="inlineStr">
         <is>
@@ -6730,11 +6724,11 @@
         </is>
       </c>
       <c r="B118" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>RARA BERKAH, CV</t>
+          <t>SATYA HARDANA, CV</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -6744,15 +6738,15 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Jl. Kancil RT.001, RW. 001 Kel. Tenilo Kec. Kota Barat</t>
+          <t>PERUM AWARA LILUWO KEC. KOTA TENGAH</t>
         </is>
       </c>
       <c r="F118" t="n">
-        <v>1933</v>
+        <v>138</v>
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>DAR AL TAUHID, CV</t>
+          <t>SATYA HARDANA, CV</t>
         </is>
       </c>
       <c r="H118" t="inlineStr">
@@ -6761,14 +6755,16 @@
         </is>
       </c>
       <c r="I118" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="J118" t="n">
         <v>100</v>
       </c>
-      <c r="K118" t="inlineStr"/>
+      <c r="K118" t="n">
+        <v>53.84615384615385</v>
+      </c>
       <c r="L118" t="n">
-        <v>60.52631578947368</v>
+        <v>71.15384615384616</v>
       </c>
       <c r="M118" t="inlineStr">
         <is>
@@ -6783,45 +6779,45 @@
         </is>
       </c>
       <c r="B119" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>FELQIMUN ADIJAYA, CV</t>
+          <t>RARA BERKAH, CV</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>7502</t>
+          <t>7571</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Jln. Brgijen Piola Isa Wongkaditi Timur Kota Utara</t>
+          <t>Jl. Kancil RT.001, RW. 001 Kel. Tenilo Kec. Kota Barat</t>
         </is>
       </c>
       <c r="F119" t="n">
-        <v>758</v>
+        <v>1933</v>
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>ADHITYA, CV</t>
+          <t>DAR AL TAUHID, CV</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>7502</t>
+          <t>7571</t>
         </is>
       </c>
       <c r="I119" t="n">
-        <v>58.06451612903225</v>
+        <v>50</v>
       </c>
       <c r="J119" t="n">
         <v>100</v>
       </c>
       <c r="K119" t="inlineStr"/>
       <c r="L119" t="n">
-        <v>65.05376344086021</v>
+        <v>60.52631578947368</v>
       </c>
       <c r="M119" t="inlineStr">
         <is>
@@ -6836,49 +6832,49 @@
         </is>
       </c>
       <c r="B120" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>ANTARIKSA PERSADA, CV</t>
+          <t>FELQIMUN ADIJAYA, CV</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>7503</t>
+          <t>7502</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Desa Sipatana Kec. Buntulia Kab. Pohuwato</t>
+          <t>Jln. Brgijen Piola Isa Wongkaditi Timur Kota Utara</t>
         </is>
       </c>
       <c r="F120" t="n">
-        <v>1226</v>
+        <v>758</v>
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>ANTARIKSA PERSADA, CV</t>
+          <t>ADHITYA, CV</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>7503</t>
+          <t>7502</t>
         </is>
       </c>
       <c r="I120" t="n">
-        <v>100</v>
+        <v>58.06451612903225</v>
       </c>
       <c r="J120" t="n">
         <v>100</v>
       </c>
       <c r="K120" t="inlineStr"/>
       <c r="L120" t="n">
-        <v>100</v>
+        <v>65.05376344086021</v>
       </c>
       <c r="M120" t="inlineStr">
         <is>
-          <t>DROP</t>
+          <t>INSERT</t>
         </is>
       </c>
     </row>
@@ -6889,49 +6885,102 @@
         </is>
       </c>
       <c r="B121" t="n">
+        <v>16</v>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>ANTARIKSA PERSADA, CV</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>7503</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Desa Sipatana Kec. Buntulia Kab. Pohuwato</t>
+        </is>
+      </c>
+      <c r="F121" t="n">
+        <v>1226</v>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>ANTARIKSA PERSADA, CV</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>7503</t>
+        </is>
+      </c>
+      <c r="I121" t="n">
+        <v>100</v>
+      </c>
+      <c r="J121" t="n">
+        <v>100</v>
+      </c>
+      <c r="K121" t="inlineStr"/>
+      <c r="L121" t="n">
+        <v>100</v>
+      </c>
+      <c r="M121" t="inlineStr">
+        <is>
+          <t>DROP</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>lpse</t>
+        </is>
+      </c>
+      <c r="B122" t="n">
         <v>17</v>
       </c>
-      <c r="C121" t="inlineStr">
+      <c r="C122" t="inlineStr">
         <is>
           <t>SEXY ROAD INDO, CV</t>
         </is>
       </c>
-      <c r="D121" t="inlineStr">
+      <c r="D122" t="inlineStr">
         <is>
           <t>7502</t>
         </is>
       </c>
-      <c r="E121" t="inlineStr">
+      <c r="E122" t="inlineStr">
         <is>
           <t>Perum Asabri Blok E no 3, Ulapato A</t>
         </is>
       </c>
-      <c r="F121" t="n">
+      <c r="F122" t="n">
         <v>55</v>
       </c>
-      <c r="G121" t="inlineStr">
+      <c r="G122" t="inlineStr">
         <is>
           <t>SEXY ROAD INDO, CV</t>
         </is>
       </c>
-      <c r="H121" t="inlineStr">
+      <c r="H122" t="inlineStr">
         <is>
           <t>7502</t>
         </is>
       </c>
-      <c r="I121" t="n">
-        <v>100</v>
-      </c>
-      <c r="J121" t="n">
-        <v>100</v>
-      </c>
-      <c r="K121" t="n">
+      <c r="I122" t="n">
+        <v>100</v>
+      </c>
+      <c r="J122" t="n">
+        <v>100</v>
+      </c>
+      <c r="K122" t="n">
         <v>77.41935483870968</v>
       </c>
-      <c r="L121" t="n">
+      <c r="L122" t="n">
         <v>86.13469156762875</v>
       </c>
-      <c r="M121" t="inlineStr">
+      <c r="M122" t="inlineStr">
         <is>
           <t>DROP</t>
         </is>

</xml_diff>